<commit_message>
awu_cran (README): add 'Metadata File' section; update sample title to 'mcars' and other updates
</commit_message>
<xml_diff>
--- a/inst/extdata/sample_titles.xlsx
+++ b/inst/extdata/sample_titles.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\GDCCTXFS002.dir.ucb-group.com\ctxctxpprd$\Redir\E643795\Documents\Amber\tflmetaR\tflmetaR\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\Sites\Braine\Biocdm\Products\MT1621\TK0117\gsp\sandbox_renv\data\misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -130,9 +130,6 @@
     <t>Table 2.1</t>
   </si>
   <si>
-    <t>Sample Table with Penguin Data</t>
-  </si>
-  <si>
     <t>Test Subtitle</t>
   </si>
   <si>
@@ -297,6 +294,9 @@
   </si>
   <si>
     <t>Data Cut-Off: 2025-12-31</t>
+  </si>
+  <si>
+    <t>Sample Table Using mtcars Data</t>
   </si>
 </sst>
 </file>
@@ -565,11 +565,11 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -959,7 +959,7 @@
         <v>24</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
@@ -1021,10 +1021,10 @@
         <v>33</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>35</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
@@ -1033,7 +1033,7 @@
         <v>24</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N4" s="21"/>
       <c r="O4" s="21"/>
@@ -1044,39 +1044,39 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L5" s="21" t="s">
         <v>24</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1095,315 +1095,315 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="29" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" style="29" customWidth="1"/>
-    <col min="3" max="4" width="11.140625" style="29" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" style="29" customWidth="1"/>
-    <col min="9" max="256" width="9.140625" style="29"/>
-    <col min="257" max="259" width="11.140625" style="29" customWidth="1"/>
-    <col min="260" max="261" width="9.140625" style="29"/>
-    <col min="262" max="264" width="11.5703125" style="29" customWidth="1"/>
-    <col min="265" max="512" width="9.140625" style="29"/>
-    <col min="513" max="515" width="11.140625" style="29" customWidth="1"/>
-    <col min="516" max="517" width="9.140625" style="29"/>
-    <col min="518" max="520" width="11.5703125" style="29" customWidth="1"/>
-    <col min="521" max="768" width="9.140625" style="29"/>
-    <col min="769" max="771" width="11.140625" style="29" customWidth="1"/>
-    <col min="772" max="773" width="9.140625" style="29"/>
-    <col min="774" max="776" width="11.5703125" style="29" customWidth="1"/>
-    <col min="777" max="1024" width="9.140625" style="29"/>
-    <col min="1025" max="1027" width="11.140625" style="29" customWidth="1"/>
-    <col min="1028" max="1029" width="9.140625" style="29"/>
-    <col min="1030" max="1032" width="11.5703125" style="29" customWidth="1"/>
-    <col min="1033" max="1280" width="9.140625" style="29"/>
-    <col min="1281" max="1283" width="11.140625" style="29" customWidth="1"/>
-    <col min="1284" max="1285" width="9.140625" style="29"/>
-    <col min="1286" max="1288" width="11.5703125" style="29" customWidth="1"/>
-    <col min="1289" max="1536" width="9.140625" style="29"/>
-    <col min="1537" max="1539" width="11.140625" style="29" customWidth="1"/>
-    <col min="1540" max="1541" width="9.140625" style="29"/>
-    <col min="1542" max="1544" width="11.5703125" style="29" customWidth="1"/>
-    <col min="1545" max="1792" width="9.140625" style="29"/>
-    <col min="1793" max="1795" width="11.140625" style="29" customWidth="1"/>
-    <col min="1796" max="1797" width="9.140625" style="29"/>
-    <col min="1798" max="1800" width="11.5703125" style="29" customWidth="1"/>
-    <col min="1801" max="2048" width="9.140625" style="29"/>
-    <col min="2049" max="2051" width="11.140625" style="29" customWidth="1"/>
-    <col min="2052" max="2053" width="9.140625" style="29"/>
-    <col min="2054" max="2056" width="11.5703125" style="29" customWidth="1"/>
-    <col min="2057" max="2304" width="9.140625" style="29"/>
-    <col min="2305" max="2307" width="11.140625" style="29" customWidth="1"/>
-    <col min="2308" max="2309" width="9.140625" style="29"/>
-    <col min="2310" max="2312" width="11.5703125" style="29" customWidth="1"/>
-    <col min="2313" max="2560" width="9.140625" style="29"/>
-    <col min="2561" max="2563" width="11.140625" style="29" customWidth="1"/>
-    <col min="2564" max="2565" width="9.140625" style="29"/>
-    <col min="2566" max="2568" width="11.5703125" style="29" customWidth="1"/>
-    <col min="2569" max="2816" width="9.140625" style="29"/>
-    <col min="2817" max="2819" width="11.140625" style="29" customWidth="1"/>
-    <col min="2820" max="2821" width="9.140625" style="29"/>
-    <col min="2822" max="2824" width="11.5703125" style="29" customWidth="1"/>
-    <col min="2825" max="3072" width="9.140625" style="29"/>
-    <col min="3073" max="3075" width="11.140625" style="29" customWidth="1"/>
-    <col min="3076" max="3077" width="9.140625" style="29"/>
-    <col min="3078" max="3080" width="11.5703125" style="29" customWidth="1"/>
-    <col min="3081" max="3328" width="9.140625" style="29"/>
-    <col min="3329" max="3331" width="11.140625" style="29" customWidth="1"/>
-    <col min="3332" max="3333" width="9.140625" style="29"/>
-    <col min="3334" max="3336" width="11.5703125" style="29" customWidth="1"/>
-    <col min="3337" max="3584" width="9.140625" style="29"/>
-    <col min="3585" max="3587" width="11.140625" style="29" customWidth="1"/>
-    <col min="3588" max="3589" width="9.140625" style="29"/>
-    <col min="3590" max="3592" width="11.5703125" style="29" customWidth="1"/>
-    <col min="3593" max="3840" width="9.140625" style="29"/>
-    <col min="3841" max="3843" width="11.140625" style="29" customWidth="1"/>
-    <col min="3844" max="3845" width="9.140625" style="29"/>
-    <col min="3846" max="3848" width="11.5703125" style="29" customWidth="1"/>
-    <col min="3849" max="4096" width="9.140625" style="29"/>
-    <col min="4097" max="4099" width="11.140625" style="29" customWidth="1"/>
-    <col min="4100" max="4101" width="9.140625" style="29"/>
-    <col min="4102" max="4104" width="11.5703125" style="29" customWidth="1"/>
-    <col min="4105" max="4352" width="9.140625" style="29"/>
-    <col min="4353" max="4355" width="11.140625" style="29" customWidth="1"/>
-    <col min="4356" max="4357" width="9.140625" style="29"/>
-    <col min="4358" max="4360" width="11.5703125" style="29" customWidth="1"/>
-    <col min="4361" max="4608" width="9.140625" style="29"/>
-    <col min="4609" max="4611" width="11.140625" style="29" customWidth="1"/>
-    <col min="4612" max="4613" width="9.140625" style="29"/>
-    <col min="4614" max="4616" width="11.5703125" style="29" customWidth="1"/>
-    <col min="4617" max="4864" width="9.140625" style="29"/>
-    <col min="4865" max="4867" width="11.140625" style="29" customWidth="1"/>
-    <col min="4868" max="4869" width="9.140625" style="29"/>
-    <col min="4870" max="4872" width="11.5703125" style="29" customWidth="1"/>
-    <col min="4873" max="5120" width="9.140625" style="29"/>
-    <col min="5121" max="5123" width="11.140625" style="29" customWidth="1"/>
-    <col min="5124" max="5125" width="9.140625" style="29"/>
-    <col min="5126" max="5128" width="11.5703125" style="29" customWidth="1"/>
-    <col min="5129" max="5376" width="9.140625" style="29"/>
-    <col min="5377" max="5379" width="11.140625" style="29" customWidth="1"/>
-    <col min="5380" max="5381" width="9.140625" style="29"/>
-    <col min="5382" max="5384" width="11.5703125" style="29" customWidth="1"/>
-    <col min="5385" max="5632" width="9.140625" style="29"/>
-    <col min="5633" max="5635" width="11.140625" style="29" customWidth="1"/>
-    <col min="5636" max="5637" width="9.140625" style="29"/>
-    <col min="5638" max="5640" width="11.5703125" style="29" customWidth="1"/>
-    <col min="5641" max="5888" width="9.140625" style="29"/>
-    <col min="5889" max="5891" width="11.140625" style="29" customWidth="1"/>
-    <col min="5892" max="5893" width="9.140625" style="29"/>
-    <col min="5894" max="5896" width="11.5703125" style="29" customWidth="1"/>
-    <col min="5897" max="6144" width="9.140625" style="29"/>
-    <col min="6145" max="6147" width="11.140625" style="29" customWidth="1"/>
-    <col min="6148" max="6149" width="9.140625" style="29"/>
-    <col min="6150" max="6152" width="11.5703125" style="29" customWidth="1"/>
-    <col min="6153" max="6400" width="9.140625" style="29"/>
-    <col min="6401" max="6403" width="11.140625" style="29" customWidth="1"/>
-    <col min="6404" max="6405" width="9.140625" style="29"/>
-    <col min="6406" max="6408" width="11.5703125" style="29" customWidth="1"/>
-    <col min="6409" max="6656" width="9.140625" style="29"/>
-    <col min="6657" max="6659" width="11.140625" style="29" customWidth="1"/>
-    <col min="6660" max="6661" width="9.140625" style="29"/>
-    <col min="6662" max="6664" width="11.5703125" style="29" customWidth="1"/>
-    <col min="6665" max="6912" width="9.140625" style="29"/>
-    <col min="6913" max="6915" width="11.140625" style="29" customWidth="1"/>
-    <col min="6916" max="6917" width="9.140625" style="29"/>
-    <col min="6918" max="6920" width="11.5703125" style="29" customWidth="1"/>
-    <col min="6921" max="7168" width="9.140625" style="29"/>
-    <col min="7169" max="7171" width="11.140625" style="29" customWidth="1"/>
-    <col min="7172" max="7173" width="9.140625" style="29"/>
-    <col min="7174" max="7176" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7177" max="7424" width="9.140625" style="29"/>
-    <col min="7425" max="7427" width="11.140625" style="29" customWidth="1"/>
-    <col min="7428" max="7429" width="9.140625" style="29"/>
-    <col min="7430" max="7432" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7433" max="7680" width="9.140625" style="29"/>
-    <col min="7681" max="7683" width="11.140625" style="29" customWidth="1"/>
-    <col min="7684" max="7685" width="9.140625" style="29"/>
-    <col min="7686" max="7688" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7689" max="7936" width="9.140625" style="29"/>
-    <col min="7937" max="7939" width="11.140625" style="29" customWidth="1"/>
-    <col min="7940" max="7941" width="9.140625" style="29"/>
-    <col min="7942" max="7944" width="11.5703125" style="29" customWidth="1"/>
-    <col min="7945" max="8192" width="9.140625" style="29"/>
-    <col min="8193" max="8195" width="11.140625" style="29" customWidth="1"/>
-    <col min="8196" max="8197" width="9.140625" style="29"/>
-    <col min="8198" max="8200" width="11.5703125" style="29" customWidth="1"/>
-    <col min="8201" max="8448" width="9.140625" style="29"/>
-    <col min="8449" max="8451" width="11.140625" style="29" customWidth="1"/>
-    <col min="8452" max="8453" width="9.140625" style="29"/>
-    <col min="8454" max="8456" width="11.5703125" style="29" customWidth="1"/>
-    <col min="8457" max="8704" width="9.140625" style="29"/>
-    <col min="8705" max="8707" width="11.140625" style="29" customWidth="1"/>
-    <col min="8708" max="8709" width="9.140625" style="29"/>
-    <col min="8710" max="8712" width="11.5703125" style="29" customWidth="1"/>
-    <col min="8713" max="8960" width="9.140625" style="29"/>
-    <col min="8961" max="8963" width="11.140625" style="29" customWidth="1"/>
-    <col min="8964" max="8965" width="9.140625" style="29"/>
-    <col min="8966" max="8968" width="11.5703125" style="29" customWidth="1"/>
-    <col min="8969" max="9216" width="9.140625" style="29"/>
-    <col min="9217" max="9219" width="11.140625" style="29" customWidth="1"/>
-    <col min="9220" max="9221" width="9.140625" style="29"/>
-    <col min="9222" max="9224" width="11.5703125" style="29" customWidth="1"/>
-    <col min="9225" max="9472" width="9.140625" style="29"/>
-    <col min="9473" max="9475" width="11.140625" style="29" customWidth="1"/>
-    <col min="9476" max="9477" width="9.140625" style="29"/>
-    <col min="9478" max="9480" width="11.5703125" style="29" customWidth="1"/>
-    <col min="9481" max="9728" width="9.140625" style="29"/>
-    <col min="9729" max="9731" width="11.140625" style="29" customWidth="1"/>
-    <col min="9732" max="9733" width="9.140625" style="29"/>
-    <col min="9734" max="9736" width="11.5703125" style="29" customWidth="1"/>
-    <col min="9737" max="9984" width="9.140625" style="29"/>
-    <col min="9985" max="9987" width="11.140625" style="29" customWidth="1"/>
-    <col min="9988" max="9989" width="9.140625" style="29"/>
-    <col min="9990" max="9992" width="11.5703125" style="29" customWidth="1"/>
-    <col min="9993" max="10240" width="9.140625" style="29"/>
-    <col min="10241" max="10243" width="11.140625" style="29" customWidth="1"/>
-    <col min="10244" max="10245" width="9.140625" style="29"/>
-    <col min="10246" max="10248" width="11.5703125" style="29" customWidth="1"/>
-    <col min="10249" max="10496" width="9.140625" style="29"/>
-    <col min="10497" max="10499" width="11.140625" style="29" customWidth="1"/>
-    <col min="10500" max="10501" width="9.140625" style="29"/>
-    <col min="10502" max="10504" width="11.5703125" style="29" customWidth="1"/>
-    <col min="10505" max="10752" width="9.140625" style="29"/>
-    <col min="10753" max="10755" width="11.140625" style="29" customWidth="1"/>
-    <col min="10756" max="10757" width="9.140625" style="29"/>
-    <col min="10758" max="10760" width="11.5703125" style="29" customWidth="1"/>
-    <col min="10761" max="11008" width="9.140625" style="29"/>
-    <col min="11009" max="11011" width="11.140625" style="29" customWidth="1"/>
-    <col min="11012" max="11013" width="9.140625" style="29"/>
-    <col min="11014" max="11016" width="11.5703125" style="29" customWidth="1"/>
-    <col min="11017" max="11264" width="9.140625" style="29"/>
-    <col min="11265" max="11267" width="11.140625" style="29" customWidth="1"/>
-    <col min="11268" max="11269" width="9.140625" style="29"/>
-    <col min="11270" max="11272" width="11.5703125" style="29" customWidth="1"/>
-    <col min="11273" max="11520" width="9.140625" style="29"/>
-    <col min="11521" max="11523" width="11.140625" style="29" customWidth="1"/>
-    <col min="11524" max="11525" width="9.140625" style="29"/>
-    <col min="11526" max="11528" width="11.5703125" style="29" customWidth="1"/>
-    <col min="11529" max="11776" width="9.140625" style="29"/>
-    <col min="11777" max="11779" width="11.140625" style="29" customWidth="1"/>
-    <col min="11780" max="11781" width="9.140625" style="29"/>
-    <col min="11782" max="11784" width="11.5703125" style="29" customWidth="1"/>
-    <col min="11785" max="12032" width="9.140625" style="29"/>
-    <col min="12033" max="12035" width="11.140625" style="29" customWidth="1"/>
-    <col min="12036" max="12037" width="9.140625" style="29"/>
-    <col min="12038" max="12040" width="11.5703125" style="29" customWidth="1"/>
-    <col min="12041" max="12288" width="9.140625" style="29"/>
-    <col min="12289" max="12291" width="11.140625" style="29" customWidth="1"/>
-    <col min="12292" max="12293" width="9.140625" style="29"/>
-    <col min="12294" max="12296" width="11.5703125" style="29" customWidth="1"/>
-    <col min="12297" max="12544" width="9.140625" style="29"/>
-    <col min="12545" max="12547" width="11.140625" style="29" customWidth="1"/>
-    <col min="12548" max="12549" width="9.140625" style="29"/>
-    <col min="12550" max="12552" width="11.5703125" style="29" customWidth="1"/>
-    <col min="12553" max="12800" width="9.140625" style="29"/>
-    <col min="12801" max="12803" width="11.140625" style="29" customWidth="1"/>
-    <col min="12804" max="12805" width="9.140625" style="29"/>
-    <col min="12806" max="12808" width="11.5703125" style="29" customWidth="1"/>
-    <col min="12809" max="13056" width="9.140625" style="29"/>
-    <col min="13057" max="13059" width="11.140625" style="29" customWidth="1"/>
-    <col min="13060" max="13061" width="9.140625" style="29"/>
-    <col min="13062" max="13064" width="11.5703125" style="29" customWidth="1"/>
-    <col min="13065" max="13312" width="9.140625" style="29"/>
-    <col min="13313" max="13315" width="11.140625" style="29" customWidth="1"/>
-    <col min="13316" max="13317" width="9.140625" style="29"/>
-    <col min="13318" max="13320" width="11.5703125" style="29" customWidth="1"/>
-    <col min="13321" max="13568" width="9.140625" style="29"/>
-    <col min="13569" max="13571" width="11.140625" style="29" customWidth="1"/>
-    <col min="13572" max="13573" width="9.140625" style="29"/>
-    <col min="13574" max="13576" width="11.5703125" style="29" customWidth="1"/>
-    <col min="13577" max="13824" width="9.140625" style="29"/>
-    <col min="13825" max="13827" width="11.140625" style="29" customWidth="1"/>
-    <col min="13828" max="13829" width="9.140625" style="29"/>
-    <col min="13830" max="13832" width="11.5703125" style="29" customWidth="1"/>
-    <col min="13833" max="14080" width="9.140625" style="29"/>
-    <col min="14081" max="14083" width="11.140625" style="29" customWidth="1"/>
-    <col min="14084" max="14085" width="9.140625" style="29"/>
-    <col min="14086" max="14088" width="11.5703125" style="29" customWidth="1"/>
-    <col min="14089" max="14336" width="9.140625" style="29"/>
-    <col min="14337" max="14339" width="11.140625" style="29" customWidth="1"/>
-    <col min="14340" max="14341" width="9.140625" style="29"/>
-    <col min="14342" max="14344" width="11.5703125" style="29" customWidth="1"/>
-    <col min="14345" max="14592" width="9.140625" style="29"/>
-    <col min="14593" max="14595" width="11.140625" style="29" customWidth="1"/>
-    <col min="14596" max="14597" width="9.140625" style="29"/>
-    <col min="14598" max="14600" width="11.5703125" style="29" customWidth="1"/>
-    <col min="14601" max="14848" width="9.140625" style="29"/>
-    <col min="14849" max="14851" width="11.140625" style="29" customWidth="1"/>
-    <col min="14852" max="14853" width="9.140625" style="29"/>
-    <col min="14854" max="14856" width="11.5703125" style="29" customWidth="1"/>
-    <col min="14857" max="15104" width="9.140625" style="29"/>
-    <col min="15105" max="15107" width="11.140625" style="29" customWidth="1"/>
-    <col min="15108" max="15109" width="9.140625" style="29"/>
-    <col min="15110" max="15112" width="11.5703125" style="29" customWidth="1"/>
-    <col min="15113" max="15360" width="9.140625" style="29"/>
-    <col min="15361" max="15363" width="11.140625" style="29" customWidth="1"/>
-    <col min="15364" max="15365" width="9.140625" style="29"/>
-    <col min="15366" max="15368" width="11.5703125" style="29" customWidth="1"/>
-    <col min="15369" max="15616" width="9.140625" style="29"/>
-    <col min="15617" max="15619" width="11.140625" style="29" customWidth="1"/>
-    <col min="15620" max="15621" width="9.140625" style="29"/>
-    <col min="15622" max="15624" width="11.5703125" style="29" customWidth="1"/>
-    <col min="15625" max="15872" width="9.140625" style="29"/>
-    <col min="15873" max="15875" width="11.140625" style="29" customWidth="1"/>
-    <col min="15876" max="15877" width="9.140625" style="29"/>
-    <col min="15878" max="15880" width="11.5703125" style="29" customWidth="1"/>
-    <col min="15881" max="16128" width="9.140625" style="29"/>
-    <col min="16129" max="16131" width="11.140625" style="29" customWidth="1"/>
-    <col min="16132" max="16133" width="9.140625" style="29"/>
-    <col min="16134" max="16136" width="11.5703125" style="29" customWidth="1"/>
-    <col min="16137" max="16384" width="9.140625" style="29"/>
+    <col min="1" max="1" width="14" style="27" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" style="27" customWidth="1"/>
+    <col min="3" max="4" width="11.140625" style="27" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" style="27" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25" style="27" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" style="27" customWidth="1"/>
+    <col min="9" max="256" width="9.140625" style="27"/>
+    <col min="257" max="259" width="11.140625" style="27" customWidth="1"/>
+    <col min="260" max="261" width="9.140625" style="27"/>
+    <col min="262" max="264" width="11.5703125" style="27" customWidth="1"/>
+    <col min="265" max="512" width="9.140625" style="27"/>
+    <col min="513" max="515" width="11.140625" style="27" customWidth="1"/>
+    <col min="516" max="517" width="9.140625" style="27"/>
+    <col min="518" max="520" width="11.5703125" style="27" customWidth="1"/>
+    <col min="521" max="768" width="9.140625" style="27"/>
+    <col min="769" max="771" width="11.140625" style="27" customWidth="1"/>
+    <col min="772" max="773" width="9.140625" style="27"/>
+    <col min="774" max="776" width="11.5703125" style="27" customWidth="1"/>
+    <col min="777" max="1024" width="9.140625" style="27"/>
+    <col min="1025" max="1027" width="11.140625" style="27" customWidth="1"/>
+    <col min="1028" max="1029" width="9.140625" style="27"/>
+    <col min="1030" max="1032" width="11.5703125" style="27" customWidth="1"/>
+    <col min="1033" max="1280" width="9.140625" style="27"/>
+    <col min="1281" max="1283" width="11.140625" style="27" customWidth="1"/>
+    <col min="1284" max="1285" width="9.140625" style="27"/>
+    <col min="1286" max="1288" width="11.5703125" style="27" customWidth="1"/>
+    <col min="1289" max="1536" width="9.140625" style="27"/>
+    <col min="1537" max="1539" width="11.140625" style="27" customWidth="1"/>
+    <col min="1540" max="1541" width="9.140625" style="27"/>
+    <col min="1542" max="1544" width="11.5703125" style="27" customWidth="1"/>
+    <col min="1545" max="1792" width="9.140625" style="27"/>
+    <col min="1793" max="1795" width="11.140625" style="27" customWidth="1"/>
+    <col min="1796" max="1797" width="9.140625" style="27"/>
+    <col min="1798" max="1800" width="11.5703125" style="27" customWidth="1"/>
+    <col min="1801" max="2048" width="9.140625" style="27"/>
+    <col min="2049" max="2051" width="11.140625" style="27" customWidth="1"/>
+    <col min="2052" max="2053" width="9.140625" style="27"/>
+    <col min="2054" max="2056" width="11.5703125" style="27" customWidth="1"/>
+    <col min="2057" max="2304" width="9.140625" style="27"/>
+    <col min="2305" max="2307" width="11.140625" style="27" customWidth="1"/>
+    <col min="2308" max="2309" width="9.140625" style="27"/>
+    <col min="2310" max="2312" width="11.5703125" style="27" customWidth="1"/>
+    <col min="2313" max="2560" width="9.140625" style="27"/>
+    <col min="2561" max="2563" width="11.140625" style="27" customWidth="1"/>
+    <col min="2564" max="2565" width="9.140625" style="27"/>
+    <col min="2566" max="2568" width="11.5703125" style="27" customWidth="1"/>
+    <col min="2569" max="2816" width="9.140625" style="27"/>
+    <col min="2817" max="2819" width="11.140625" style="27" customWidth="1"/>
+    <col min="2820" max="2821" width="9.140625" style="27"/>
+    <col min="2822" max="2824" width="11.5703125" style="27" customWidth="1"/>
+    <col min="2825" max="3072" width="9.140625" style="27"/>
+    <col min="3073" max="3075" width="11.140625" style="27" customWidth="1"/>
+    <col min="3076" max="3077" width="9.140625" style="27"/>
+    <col min="3078" max="3080" width="11.5703125" style="27" customWidth="1"/>
+    <col min="3081" max="3328" width="9.140625" style="27"/>
+    <col min="3329" max="3331" width="11.140625" style="27" customWidth="1"/>
+    <col min="3332" max="3333" width="9.140625" style="27"/>
+    <col min="3334" max="3336" width="11.5703125" style="27" customWidth="1"/>
+    <col min="3337" max="3584" width="9.140625" style="27"/>
+    <col min="3585" max="3587" width="11.140625" style="27" customWidth="1"/>
+    <col min="3588" max="3589" width="9.140625" style="27"/>
+    <col min="3590" max="3592" width="11.5703125" style="27" customWidth="1"/>
+    <col min="3593" max="3840" width="9.140625" style="27"/>
+    <col min="3841" max="3843" width="11.140625" style="27" customWidth="1"/>
+    <col min="3844" max="3845" width="9.140625" style="27"/>
+    <col min="3846" max="3848" width="11.5703125" style="27" customWidth="1"/>
+    <col min="3849" max="4096" width="9.140625" style="27"/>
+    <col min="4097" max="4099" width="11.140625" style="27" customWidth="1"/>
+    <col min="4100" max="4101" width="9.140625" style="27"/>
+    <col min="4102" max="4104" width="11.5703125" style="27" customWidth="1"/>
+    <col min="4105" max="4352" width="9.140625" style="27"/>
+    <col min="4353" max="4355" width="11.140625" style="27" customWidth="1"/>
+    <col min="4356" max="4357" width="9.140625" style="27"/>
+    <col min="4358" max="4360" width="11.5703125" style="27" customWidth="1"/>
+    <col min="4361" max="4608" width="9.140625" style="27"/>
+    <col min="4609" max="4611" width="11.140625" style="27" customWidth="1"/>
+    <col min="4612" max="4613" width="9.140625" style="27"/>
+    <col min="4614" max="4616" width="11.5703125" style="27" customWidth="1"/>
+    <col min="4617" max="4864" width="9.140625" style="27"/>
+    <col min="4865" max="4867" width="11.140625" style="27" customWidth="1"/>
+    <col min="4868" max="4869" width="9.140625" style="27"/>
+    <col min="4870" max="4872" width="11.5703125" style="27" customWidth="1"/>
+    <col min="4873" max="5120" width="9.140625" style="27"/>
+    <col min="5121" max="5123" width="11.140625" style="27" customWidth="1"/>
+    <col min="5124" max="5125" width="9.140625" style="27"/>
+    <col min="5126" max="5128" width="11.5703125" style="27" customWidth="1"/>
+    <col min="5129" max="5376" width="9.140625" style="27"/>
+    <col min="5377" max="5379" width="11.140625" style="27" customWidth="1"/>
+    <col min="5380" max="5381" width="9.140625" style="27"/>
+    <col min="5382" max="5384" width="11.5703125" style="27" customWidth="1"/>
+    <col min="5385" max="5632" width="9.140625" style="27"/>
+    <col min="5633" max="5635" width="11.140625" style="27" customWidth="1"/>
+    <col min="5636" max="5637" width="9.140625" style="27"/>
+    <col min="5638" max="5640" width="11.5703125" style="27" customWidth="1"/>
+    <col min="5641" max="5888" width="9.140625" style="27"/>
+    <col min="5889" max="5891" width="11.140625" style="27" customWidth="1"/>
+    <col min="5892" max="5893" width="9.140625" style="27"/>
+    <col min="5894" max="5896" width="11.5703125" style="27" customWidth="1"/>
+    <col min="5897" max="6144" width="9.140625" style="27"/>
+    <col min="6145" max="6147" width="11.140625" style="27" customWidth="1"/>
+    <col min="6148" max="6149" width="9.140625" style="27"/>
+    <col min="6150" max="6152" width="11.5703125" style="27" customWidth="1"/>
+    <col min="6153" max="6400" width="9.140625" style="27"/>
+    <col min="6401" max="6403" width="11.140625" style="27" customWidth="1"/>
+    <col min="6404" max="6405" width="9.140625" style="27"/>
+    <col min="6406" max="6408" width="11.5703125" style="27" customWidth="1"/>
+    <col min="6409" max="6656" width="9.140625" style="27"/>
+    <col min="6657" max="6659" width="11.140625" style="27" customWidth="1"/>
+    <col min="6660" max="6661" width="9.140625" style="27"/>
+    <col min="6662" max="6664" width="11.5703125" style="27" customWidth="1"/>
+    <col min="6665" max="6912" width="9.140625" style="27"/>
+    <col min="6913" max="6915" width="11.140625" style="27" customWidth="1"/>
+    <col min="6916" max="6917" width="9.140625" style="27"/>
+    <col min="6918" max="6920" width="11.5703125" style="27" customWidth="1"/>
+    <col min="6921" max="7168" width="9.140625" style="27"/>
+    <col min="7169" max="7171" width="11.140625" style="27" customWidth="1"/>
+    <col min="7172" max="7173" width="9.140625" style="27"/>
+    <col min="7174" max="7176" width="11.5703125" style="27" customWidth="1"/>
+    <col min="7177" max="7424" width="9.140625" style="27"/>
+    <col min="7425" max="7427" width="11.140625" style="27" customWidth="1"/>
+    <col min="7428" max="7429" width="9.140625" style="27"/>
+    <col min="7430" max="7432" width="11.5703125" style="27" customWidth="1"/>
+    <col min="7433" max="7680" width="9.140625" style="27"/>
+    <col min="7681" max="7683" width="11.140625" style="27" customWidth="1"/>
+    <col min="7684" max="7685" width="9.140625" style="27"/>
+    <col min="7686" max="7688" width="11.5703125" style="27" customWidth="1"/>
+    <col min="7689" max="7936" width="9.140625" style="27"/>
+    <col min="7937" max="7939" width="11.140625" style="27" customWidth="1"/>
+    <col min="7940" max="7941" width="9.140625" style="27"/>
+    <col min="7942" max="7944" width="11.5703125" style="27" customWidth="1"/>
+    <col min="7945" max="8192" width="9.140625" style="27"/>
+    <col min="8193" max="8195" width="11.140625" style="27" customWidth="1"/>
+    <col min="8196" max="8197" width="9.140625" style="27"/>
+    <col min="8198" max="8200" width="11.5703125" style="27" customWidth="1"/>
+    <col min="8201" max="8448" width="9.140625" style="27"/>
+    <col min="8449" max="8451" width="11.140625" style="27" customWidth="1"/>
+    <col min="8452" max="8453" width="9.140625" style="27"/>
+    <col min="8454" max="8456" width="11.5703125" style="27" customWidth="1"/>
+    <col min="8457" max="8704" width="9.140625" style="27"/>
+    <col min="8705" max="8707" width="11.140625" style="27" customWidth="1"/>
+    <col min="8708" max="8709" width="9.140625" style="27"/>
+    <col min="8710" max="8712" width="11.5703125" style="27" customWidth="1"/>
+    <col min="8713" max="8960" width="9.140625" style="27"/>
+    <col min="8961" max="8963" width="11.140625" style="27" customWidth="1"/>
+    <col min="8964" max="8965" width="9.140625" style="27"/>
+    <col min="8966" max="8968" width="11.5703125" style="27" customWidth="1"/>
+    <col min="8969" max="9216" width="9.140625" style="27"/>
+    <col min="9217" max="9219" width="11.140625" style="27" customWidth="1"/>
+    <col min="9220" max="9221" width="9.140625" style="27"/>
+    <col min="9222" max="9224" width="11.5703125" style="27" customWidth="1"/>
+    <col min="9225" max="9472" width="9.140625" style="27"/>
+    <col min="9473" max="9475" width="11.140625" style="27" customWidth="1"/>
+    <col min="9476" max="9477" width="9.140625" style="27"/>
+    <col min="9478" max="9480" width="11.5703125" style="27" customWidth="1"/>
+    <col min="9481" max="9728" width="9.140625" style="27"/>
+    <col min="9729" max="9731" width="11.140625" style="27" customWidth="1"/>
+    <col min="9732" max="9733" width="9.140625" style="27"/>
+    <col min="9734" max="9736" width="11.5703125" style="27" customWidth="1"/>
+    <col min="9737" max="9984" width="9.140625" style="27"/>
+    <col min="9985" max="9987" width="11.140625" style="27" customWidth="1"/>
+    <col min="9988" max="9989" width="9.140625" style="27"/>
+    <col min="9990" max="9992" width="11.5703125" style="27" customWidth="1"/>
+    <col min="9993" max="10240" width="9.140625" style="27"/>
+    <col min="10241" max="10243" width="11.140625" style="27" customWidth="1"/>
+    <col min="10244" max="10245" width="9.140625" style="27"/>
+    <col min="10246" max="10248" width="11.5703125" style="27" customWidth="1"/>
+    <col min="10249" max="10496" width="9.140625" style="27"/>
+    <col min="10497" max="10499" width="11.140625" style="27" customWidth="1"/>
+    <col min="10500" max="10501" width="9.140625" style="27"/>
+    <col min="10502" max="10504" width="11.5703125" style="27" customWidth="1"/>
+    <col min="10505" max="10752" width="9.140625" style="27"/>
+    <col min="10753" max="10755" width="11.140625" style="27" customWidth="1"/>
+    <col min="10756" max="10757" width="9.140625" style="27"/>
+    <col min="10758" max="10760" width="11.5703125" style="27" customWidth="1"/>
+    <col min="10761" max="11008" width="9.140625" style="27"/>
+    <col min="11009" max="11011" width="11.140625" style="27" customWidth="1"/>
+    <col min="11012" max="11013" width="9.140625" style="27"/>
+    <col min="11014" max="11016" width="11.5703125" style="27" customWidth="1"/>
+    <col min="11017" max="11264" width="9.140625" style="27"/>
+    <col min="11265" max="11267" width="11.140625" style="27" customWidth="1"/>
+    <col min="11268" max="11269" width="9.140625" style="27"/>
+    <col min="11270" max="11272" width="11.5703125" style="27" customWidth="1"/>
+    <col min="11273" max="11520" width="9.140625" style="27"/>
+    <col min="11521" max="11523" width="11.140625" style="27" customWidth="1"/>
+    <col min="11524" max="11525" width="9.140625" style="27"/>
+    <col min="11526" max="11528" width="11.5703125" style="27" customWidth="1"/>
+    <col min="11529" max="11776" width="9.140625" style="27"/>
+    <col min="11777" max="11779" width="11.140625" style="27" customWidth="1"/>
+    <col min="11780" max="11781" width="9.140625" style="27"/>
+    <col min="11782" max="11784" width="11.5703125" style="27" customWidth="1"/>
+    <col min="11785" max="12032" width="9.140625" style="27"/>
+    <col min="12033" max="12035" width="11.140625" style="27" customWidth="1"/>
+    <col min="12036" max="12037" width="9.140625" style="27"/>
+    <col min="12038" max="12040" width="11.5703125" style="27" customWidth="1"/>
+    <col min="12041" max="12288" width="9.140625" style="27"/>
+    <col min="12289" max="12291" width="11.140625" style="27" customWidth="1"/>
+    <col min="12292" max="12293" width="9.140625" style="27"/>
+    <col min="12294" max="12296" width="11.5703125" style="27" customWidth="1"/>
+    <col min="12297" max="12544" width="9.140625" style="27"/>
+    <col min="12545" max="12547" width="11.140625" style="27" customWidth="1"/>
+    <col min="12548" max="12549" width="9.140625" style="27"/>
+    <col min="12550" max="12552" width="11.5703125" style="27" customWidth="1"/>
+    <col min="12553" max="12800" width="9.140625" style="27"/>
+    <col min="12801" max="12803" width="11.140625" style="27" customWidth="1"/>
+    <col min="12804" max="12805" width="9.140625" style="27"/>
+    <col min="12806" max="12808" width="11.5703125" style="27" customWidth="1"/>
+    <col min="12809" max="13056" width="9.140625" style="27"/>
+    <col min="13057" max="13059" width="11.140625" style="27" customWidth="1"/>
+    <col min="13060" max="13061" width="9.140625" style="27"/>
+    <col min="13062" max="13064" width="11.5703125" style="27" customWidth="1"/>
+    <col min="13065" max="13312" width="9.140625" style="27"/>
+    <col min="13313" max="13315" width="11.140625" style="27" customWidth="1"/>
+    <col min="13316" max="13317" width="9.140625" style="27"/>
+    <col min="13318" max="13320" width="11.5703125" style="27" customWidth="1"/>
+    <col min="13321" max="13568" width="9.140625" style="27"/>
+    <col min="13569" max="13571" width="11.140625" style="27" customWidth="1"/>
+    <col min="13572" max="13573" width="9.140625" style="27"/>
+    <col min="13574" max="13576" width="11.5703125" style="27" customWidth="1"/>
+    <col min="13577" max="13824" width="9.140625" style="27"/>
+    <col min="13825" max="13827" width="11.140625" style="27" customWidth="1"/>
+    <col min="13828" max="13829" width="9.140625" style="27"/>
+    <col min="13830" max="13832" width="11.5703125" style="27" customWidth="1"/>
+    <col min="13833" max="14080" width="9.140625" style="27"/>
+    <col min="14081" max="14083" width="11.140625" style="27" customWidth="1"/>
+    <col min="14084" max="14085" width="9.140625" style="27"/>
+    <col min="14086" max="14088" width="11.5703125" style="27" customWidth="1"/>
+    <col min="14089" max="14336" width="9.140625" style="27"/>
+    <col min="14337" max="14339" width="11.140625" style="27" customWidth="1"/>
+    <col min="14340" max="14341" width="9.140625" style="27"/>
+    <col min="14342" max="14344" width="11.5703125" style="27" customWidth="1"/>
+    <col min="14345" max="14592" width="9.140625" style="27"/>
+    <col min="14593" max="14595" width="11.140625" style="27" customWidth="1"/>
+    <col min="14596" max="14597" width="9.140625" style="27"/>
+    <col min="14598" max="14600" width="11.5703125" style="27" customWidth="1"/>
+    <col min="14601" max="14848" width="9.140625" style="27"/>
+    <col min="14849" max="14851" width="11.140625" style="27" customWidth="1"/>
+    <col min="14852" max="14853" width="9.140625" style="27"/>
+    <col min="14854" max="14856" width="11.5703125" style="27" customWidth="1"/>
+    <col min="14857" max="15104" width="9.140625" style="27"/>
+    <col min="15105" max="15107" width="11.140625" style="27" customWidth="1"/>
+    <col min="15108" max="15109" width="9.140625" style="27"/>
+    <col min="15110" max="15112" width="11.5703125" style="27" customWidth="1"/>
+    <col min="15113" max="15360" width="9.140625" style="27"/>
+    <col min="15361" max="15363" width="11.140625" style="27" customWidth="1"/>
+    <col min="15364" max="15365" width="9.140625" style="27"/>
+    <col min="15366" max="15368" width="11.5703125" style="27" customWidth="1"/>
+    <col min="15369" max="15616" width="9.140625" style="27"/>
+    <col min="15617" max="15619" width="11.140625" style="27" customWidth="1"/>
+    <col min="15620" max="15621" width="9.140625" style="27"/>
+    <col min="15622" max="15624" width="11.5703125" style="27" customWidth="1"/>
+    <col min="15625" max="15872" width="9.140625" style="27"/>
+    <col min="15873" max="15875" width="11.140625" style="27" customWidth="1"/>
+    <col min="15876" max="15877" width="9.140625" style="27"/>
+    <col min="15878" max="15880" width="11.5703125" style="27" customWidth="1"/>
+    <col min="15881" max="16128" width="9.140625" style="27"/>
+    <col min="16129" max="16131" width="11.140625" style="27" customWidth="1"/>
+    <col min="16132" max="16133" width="9.140625" style="27"/>
+    <col min="16134" max="16136" width="11.5703125" style="27" customWidth="1"/>
+    <col min="16137" max="16384" width="9.140625" style="27"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="C1" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="D1" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="E1" s="29" t="s">
         <v>75</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="F1" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="F1" s="31" t="s">
+      <c r="G1" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="H1" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="H1" s="31" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A2" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="28" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="30" t="s">
+      <c r="C2" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="D2" s="28"/>
+      <c r="E2" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="F2" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="G2" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30" t="s">
-        <v>81</v>
-      </c>
-      <c r="F2" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="H2" s="30"/>
+      <c r="H2" s="28"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1906,42 +1906,42 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>46</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="9"/>
       <c r="B2" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="11"/>
       <c r="B3" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="12"/>
       <c r="B4" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="13"/>
       <c r="B5" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>52</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1949,10 +1949,10 @@
         <v>1</v>
       </c>
       <c r="B8" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="30" t="s">
         <v>54</v>
-      </c>
-      <c r="C8" s="27" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1960,32 +1960,32 @@
         <v>2</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="28"/>
+        <v>55</v>
+      </c>
+      <c r="C9" s="31"/>
     </row>
     <row r="10" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="19" t="s">
         <v>60</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -1993,7 +1993,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
@@ -2001,7 +2001,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -2009,7 +2009,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C15" s="10"/>
     </row>
@@ -2018,7 +2018,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="25.5" x14ac:dyDescent="0.2">
@@ -2026,7 +2026,7 @@
         <v>11</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="25.5" x14ac:dyDescent="0.2">
@@ -2034,22 +2034,22 @@
         <v>12</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B22" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B23" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B24" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>